<commit_message>
Add tier-grouped ranking sheet to workbook
</commit_message>
<xml_diff>
--- a/examples/example_model.xlsx
+++ b/examples/example_model.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Market_Offers" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Scenario_Model" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Backtest" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Recommendation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tier_Ranking" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Recommendation" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,7 +63,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -152,6 +158,20 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5929,6 +5949,676 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Tier_Ranking — decide commit-to-a-price vs follow-the-market FIRST, then compare within the tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Floating, 1-year fixed and multi-year fixed are different RISK products, not one price line. Per supply, offers are grouped by commitment tier and ranked cheapest-first WITHIN each tier (computed on the sampled bills; re-run the builder after editing Market_Offers). Weigh the fixed term: a long lock in a volatile market is opportunity risk + an exit fee, not free certainty. Cheapest in each tier is highlighted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>D1 — DEMO — Main residence (night tariff)  ·  current actual (sample): €538.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Eff. €/kWh</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>New total (sample) €</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Saving €</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Saving %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="22" t="inlineStr">
+        <is>
+          <t>Floating — follow the market</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n"/>
+      <c r="C6" s="23" t="n"/>
+      <c r="D6" s="23" t="n"/>
+      <c r="E6" s="23" t="n"/>
+      <c r="F6" s="23" t="n"/>
+      <c r="G6" s="23" t="n"/>
+      <c r="H6" s="23" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Floating Night (demo)</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Provider-C</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>0.1133</v>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>463.95</v>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>74.12</v>
+      </c>
+      <c r="H7" s="27" t="n">
+        <v>0.1377538858017234</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Cost+ Home (demo)</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Provider-C</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>491.86</v>
+      </c>
+      <c r="G8" s="12" t="n">
+        <v>46.21</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>0.08587383302048664</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Zero-Paygio Home (demo)</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Provider-D</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>501.37</v>
+      </c>
+      <c r="G9" s="12" t="n">
+        <v>36.7</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>0.06821603137138278</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>Fixed ≤ 12 months</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n"/>
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="23" t="n"/>
+      <c r="E10" s="23" t="n"/>
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="23" t="n"/>
+      <c r="H10" s="23" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>Fixed Home 12M (demo)</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Provider-E</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>12 months fixed</t>
+        </is>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>533.04</v>
+      </c>
+      <c r="G11" s="26" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>0.009352314754585605</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>Fixed 13–24 months</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n"/>
+      <c r="C12" s="23" t="n"/>
+      <c r="D12" s="23" t="n"/>
+      <c r="E12" s="23" t="n"/>
+      <c r="F12" s="23" t="n"/>
+      <c r="G12" s="23" t="n"/>
+      <c r="H12" s="23" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>Fixed Night 24M (demo)</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Provider-A</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>24 months fixed</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>0.145</v>
+      </c>
+      <c r="F13" s="26" t="n">
+        <v>521.88</v>
+      </c>
+      <c r="G13" s="26" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="H13" s="27" t="n">
+        <v>0.03009645585146907</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>D2 — DEMO — Apartment  ·  current actual (sample): €159.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Eff. €/kWh</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>New total (sample) €</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Saving €</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Saving %</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>Floating — follow the market</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="23" t="n"/>
+      <c r="D17" s="23" t="n"/>
+      <c r="E17" s="23" t="n"/>
+      <c r="F17" s="23" t="n"/>
+      <c r="G17" s="23" t="n"/>
+      <c r="H17" s="23" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Zero-Paygio Home (demo)</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>Provider-D</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="F18" s="26" t="n">
+        <v>134.06</v>
+      </c>
+      <c r="G18" s="26" t="n">
+        <v>25.93</v>
+      </c>
+      <c r="H18" s="27" t="n">
+        <v>0.1620451278204888</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Cost+ Home (demo)</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Provider-C</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>141.93</v>
+      </c>
+      <c r="G19" s="12" t="n">
+        <v>18.06</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>0.1129066399983333</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>Fixed ≤ 12 months</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="23" t="n"/>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="23" t="n"/>
+      <c r="G20" s="23" t="n"/>
+      <c r="H20" s="23" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Fixed Home 12M (demo)</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Provider-E</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>12 months fixed</t>
+        </is>
+      </c>
+      <c r="E21" s="25" t="n">
+        <v>0.139</v>
+      </c>
+      <c r="F21" s="26" t="n">
+        <v>158.5</v>
+      </c>
+      <c r="G21" s="26" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="H21" s="27" t="n">
+        <v>0.009296206012875834</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>D3 — DEMO — Building common areas  ·  current actual (sample): €381.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Term</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Eff. €/kWh</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>New total (sample) €</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Saving €</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Saving %</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>Floating — follow the market</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="23" t="n"/>
+      <c r="G25" s="23" t="n"/>
+      <c r="H25" s="23" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="24" t="inlineStr">
+        <is>
+          <t>Business Green (demo)</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Provider-D</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E26" s="25" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="F26" s="26" t="n">
+        <v>295.73</v>
+      </c>
+      <c r="G26" s="26" t="n">
+        <v>85.86</v>
+      </c>
+      <c r="H26" s="27" t="n">
+        <v>0.2250027516444352</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Business Saver (demo)</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>Provider-B</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="n">
+        <v>0.133</v>
+      </c>
+      <c r="F27" s="12" t="n">
+        <v>329.85</v>
+      </c>
+      <c r="G27" s="12" t="n">
+        <v>51.74</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>0.1356022607161263</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>Fixed ≤ 12 months</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="23" t="n"/>
+      <c r="G28" s="23" t="n"/>
+      <c r="H28" s="23" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Business Fixed 12M (demo)</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Provider-E</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>12 months fixed</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="F29" s="26" t="n">
+        <v>402.86</v>
+      </c>
+      <c r="G29" s="26" t="n">
+        <v>-21.27</v>
+      </c>
+      <c r="H29" s="27" t="n">
+        <v>-0.05573608672484439</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A10:H10"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A17:H17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6106,7 +6796,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Overall expected savings: see Backtest TOTAL row. Headline figures are summarised in the report.</t>
         </is>

</xml_diff>

<commit_message>
Unify tier and backtest logic in engine; builders import it
</commit_message>
<xml_diff>
--- a/examples/example_model.xlsx
+++ b/examples/example_model.xlsx
@@ -5972,7 +5972,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Floating, 1-year fixed and multi-year fixed are different RISK products, not one price line. Per supply, offers are grouped by commitment tier and ranked cheapest-first WITHIN each tier (computed on the sampled bills; re-run the builder after editing Market_Offers). Weigh the fixed term: a long lock in a volatile market is opportunity risk + an exit fee, not free certainty. Cheapest in each tier is highlighted.</t>
+          <t>Floating, 1-year fixed and multi-year fixed are different RISK products, not one price line. Per supply, offers are grouped by commitment tier and ranked cheapest-first WITHIN each tier (computed on the sampled bills; re-run the builder after editing Market_Offers). Weigh the fixed term: a long lock in a volatile market is opportunity risk + an exit fee, not free certainty. Cheapest in each tier is highlighted. Tier classification + backtest come from backtest_engine.py (single source of truth).</t>
         </is>
       </c>
     </row>
@@ -6070,7 +6070,7 @@
         <v>74.12</v>
       </c>
       <c r="H7" s="27" t="n">
-        <v>0.1377538858017234</v>
+        <v>0.1377515936588176</v>
       </c>
     </row>
     <row r="8">
@@ -6104,7 +6104,7 @@
         <v>46.21</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>0.08587383302048664</v>
+        <v>0.08588101919824558</v>
       </c>
     </row>
     <row r="9">
@@ -6132,13 +6132,13 @@
         <v>0.134</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>501.37</v>
+        <v>501.36</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>36.7</v>
+        <v>36.71</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>0.06821603137138278</v>
+        <v>0.0682253238426227</v>
       </c>
     </row>
     <row r="10">
@@ -6186,7 +6186,7 @@
         <v>5.03</v>
       </c>
       <c r="H11" s="27" t="n">
-        <v>0.009352314754585605</v>
+        <v>0.009348226067240322</v>
       </c>
     </row>
     <row r="12">
@@ -6234,7 +6234,7 @@
         <v>16.19</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>0.03009645585146907</v>
+        <v>0.0300890218744773</v>
       </c>
     </row>
     <row r="15">
@@ -6325,13 +6325,13 @@
         <v>0.134</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>134.06</v>
+        <v>134.07</v>
       </c>
       <c r="G18" s="26" t="n">
-        <v>25.93</v>
+        <v>25.92</v>
       </c>
       <c r="H18" s="27" t="n">
-        <v>0.1620451278204888</v>
+        <v>0.1620101256328521</v>
       </c>
     </row>
     <row r="19">
@@ -6365,7 +6365,7 @@
         <v>18.06</v>
       </c>
       <c r="H19" s="16" t="n">
-        <v>0.1129066399983333</v>
+        <v>0.1128820551284455</v>
       </c>
     </row>
     <row r="20">
@@ -6413,7 +6413,7 @@
         <v>1.49</v>
       </c>
       <c r="H21" s="27" t="n">
-        <v>0.009296206012875834</v>
+        <v>0.009313082067629225</v>
       </c>
     </row>
     <row r="23">
@@ -6510,7 +6510,7 @@
         <v>85.86</v>
       </c>
       <c r="H26" s="27" t="n">
-        <v>0.2250027516444352</v>
+        <v>0.2250058963809324</v>
       </c>
     </row>
     <row r="27">
@@ -6538,13 +6538,13 @@
         <v>0.133</v>
       </c>
       <c r="F27" s="12" t="n">
-        <v>329.85</v>
+        <v>329.84</v>
       </c>
       <c r="G27" s="12" t="n">
-        <v>51.74</v>
+        <v>51.75</v>
       </c>
       <c r="H27" s="16" t="n">
-        <v>0.1356022607161263</v>
+        <v>0.1356167614455306</v>
       </c>
     </row>
     <row r="28">
@@ -6592,7 +6592,7 @@
         <v>-21.27</v>
       </c>
       <c r="H29" s="27" t="n">
-        <v>-0.05573608672484439</v>
+        <v>-0.05574045441442386</v>
       </c>
     </row>
   </sheetData>

</xml_diff>